<commit_message>
Deep-link permit request numbers to the municipality file view (closes #96) (#97)
Each מספר בקשה in the permits table now links to the file in the
municipality licensing viewer:
#/Details?TikNum=<num>&SystemCode=26400046&Page=BakashalInfo
(תיק רישוי בניה). Pattern verified against the SPA's own router and nav
links (Wayback copy of its JS bundle), a production referrer using the
same pattern, and a live browser session where the page loaded and
auto-fetched proc 242700447 for the URL's tik. Section note updated.

Co-authored-by: planning-watch agent <agent@local>
</commit_message>
<xml_diff>
--- a/out/ginot_hair_plans.xlsx
+++ b/out/ginot_hair_plans.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="plans" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="counts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plans" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>